<commit_message>
Adding top results and rationale
</commit_message>
<xml_diff>
--- a/docs/downloads/top_results.xlsx
+++ b/docs/downloads/top_results.xlsx
@@ -59,6 +59,27 @@
     <t xml:space="preserve">DHHS</t>
   </si>
   <si>
+    <t xml:space="preserve">CDC-RFA-PS-27-0009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrated Viral Hepatitis Surveillance, Testing, Treatment, and Prevention Programs for Health Departments (IVH-STTP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HHS-CDC-NCHHSTP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forecasted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 139 days to deadline · about $7.5M per award (estimated: total ÷ expected awards) · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No escalation: required capabilities are in-house or contracted, no cost share, about 0.5 FTE fits your staff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/2e580529-c869-47d0-9aab-7d0e239ed5e8</t>
+  </si>
+  <si>
     <t xml:space="preserve">HRSA-27-007</t>
   </si>
   <si>
@@ -68,9 +89,6 @@
     <t xml:space="preserve">HHS-HRSA</t>
   </si>
   <si>
-    <t xml:space="preserve">forecasted</t>
-  </si>
-  <si>
     <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 91 days to deadline · up to $22.0M (Grants.gov ceiling) · no cost share → Tier 1: writer can act</t>
   </si>
   <si>
@@ -80,22 +98,16 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/c30fddfd-2094-4cf0-ba21-04b6736fc755</t>
   </si>
   <si>
-    <t xml:space="preserve">CDC-RFA-PS-27-0009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integrated Viral Hepatitis Surveillance, Testing, Treatment, and Prevention Programs for Health Departments (IVH-STTP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HHS-CDC-NCHHSTP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 139 days to deadline · award not stated on Grants.gov · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No escalation: required capabilities are in-house or contracted, no cost share, about 0.5 FTE fits your staff</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/2e580529-c869-47d0-9aab-7d0e239ed5e8</t>
+    <t xml:space="preserve">HRSA-27-006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiscal Year (FY) 2027 Service Area Competition (SAC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 91 days to deadline · up to $19.2M (Grants.gov ceiling) · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/51fa7e21-beca-497f-a0f1-bf175382f77f</t>
   </si>
   <si>
     <t xml:space="preserve">CDC-RFA-CK-27-0007</t>
@@ -113,18 +125,6 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/38e79010-c2a9-4d5f-bf81-cede591318e4</t>
   </si>
   <si>
-    <t xml:space="preserve">HRSA-27-006</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fiscal Year (FY) 2027 Service Area Competition (SAC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 91 days to deadline · up to $19.2M (Grants.gov ceiling) · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/51fa7e21-beca-497f-a0f1-bf175382f77f</t>
-  </si>
-  <si>
     <t xml:space="preserve">HRSA-27-008</t>
   </si>
   <si>
@@ -146,6 +146,42 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/be465a8b-8694-4eef-9801-5160a92c7cdf</t>
   </si>
   <si>
+    <t xml:space="preserve">CDC-RFA-PS-27-0008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Controlling and Preventing STIs in US Health Departments (CAP-STIs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 103 days to deadline · about $8.5M per award (estimated: total ÷ expected awards) · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/0ff3ace3-70fb-4ef7-b6ba-b93a899a2707</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CDC-RFA-PS-27-0239</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Strengthening Services to Prevent the Infectious Disease Consequences of Drug Use</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 236 days to deadline · about $41.2M per award (estimated: total ÷ expected awards) · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/441d2761-0d9c-42ae-a3da-905ce4ed0ca4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRSA-27-063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HIV Care Grant Program - Part B States/Territories Formula and AIDS Drug Assistance Program Formula and AIDS Drug Assistance Program Supplemental Awards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 92 days to deadline · about $21.7M per award (estimated: total ÷ expected awards) · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/1d55627c-531e-4a60-95e0-719b256179bf</t>
+  </si>
+  <si>
     <t xml:space="preserve">HRSA-27-077</t>
   </si>
   <si>
@@ -170,6 +206,45 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/d9551b09-3a45-4dc1-a343-3f09521de9aa</t>
   </si>
   <si>
+    <t xml:space="preserve">CDC-RFA-DD-27-0065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surveillance and Case Control Study of Stillbirth and Birth Defects (SUCCSSBD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HHS-CDC-NCBDDD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 182 days to deadline · about $2.8M per award (estimated: total ÷ expected awards) · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/91d0d477-b844-4189-8880-bd7a2876b24e</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CDC-RFA-PS-27-0237</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Holistic and Evidence-Informed Wellness for STI Prevention</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 243 days to deadline · about $3.0M per award (estimated: total ÷ expected awards) · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/e511b41d-655a-4869-bfd3-09fbf0c33987</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CDC-RFA-DD-27-0028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maternal-Child Surveillance and Partnerships for Action, Results, and Knowledge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 208 days to deadline · about $2.2M per award (estimated: total ÷ expected awards) · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/172926e9-5f18-4993-893d-ac73be5bbb9d</t>
+  </si>
+  <si>
     <t xml:space="preserve">RFA-IP-27-035</t>
   </si>
   <si>
@@ -185,6 +260,21 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/b3577f33-eee0-49fb-aeba-2ea0b02fe59e</t>
   </si>
   <si>
+    <t xml:space="preserve">FOR-FD-23-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manufactured Foods Flexible Funding Model (MF-FFM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HHS-FDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · no deadline stated · award not stated on Grants.gov · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/b8b51aae-68fc-448a-bbca-5fbfd229a841</t>
+  </si>
+  <si>
     <t xml:space="preserve">HRSA-27-019</t>
   </si>
   <si>
@@ -221,18 +311,6 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/741f2935-18c1-4e3e-8f54-f30dc3a6ee80</t>
   </si>
   <si>
-    <t xml:space="preserve">CDC-RFA-PS-27-0008</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Controlling and Preventing STIs in US Health Departments (CAP-STIs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 103 days to deadline · award not stated on Grants.gov · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/0ff3ace3-70fb-4ef7-b6ba-b93a899a2707</t>
-  </si>
-  <si>
     <t xml:space="preserve">HRSA-27-046</t>
   </si>
   <si>
@@ -245,58 +323,16 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/6bc69d9c-87b7-4329-962c-16c8e3ad553d</t>
   </si>
   <si>
-    <t xml:space="preserve">CDC-RFA-DD-27-0065</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Surveillance and Case Control Study of Stillbirth and Birth Defects (SUCCSSBD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HHS-CDC-NCBDDD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 182 days to deadline · award not stated on Grants.gov · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/91d0d477-b844-4189-8880-bd7a2876b24e</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CDC-RFA-DD-27-0028</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maternal-Child Surveillance and Partnerships for Action, Results, and Knowledge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 208 days to deadline · award not stated on Grants.gov · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/172926e9-5f18-4993-893d-ac73be5bbb9d</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CDC-RFA-PS-27-0237</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holistic and Evidence-Informed Wellness for STI Prevention</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 243 days to deadline · award not stated on Grants.gov · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/e511b41d-655a-4869-bfd3-09fbf0c33987</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOR-FD-23-014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Manufactured Foods Flexible Funding Model (MF-FFM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HHS-FDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · no deadline stated · award not stated on Grants.gov · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/b8b51aae-68fc-448a-bbca-5fbfd229a841</t>
+    <t xml:space="preserve">HRSA-27-079</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ryan White HIV/AIDS Program (RWHAP) Integrated HIV/AIDS Planning Resource Allocation Cooperative Agreement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 110 days to deadline · up to $700K (Grants.gov ceiling) · no cost share → Tier 1: writer can act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/a73919b2-7a90-4735-8ec5-a67c08dea3ed</t>
   </si>
   <si>
     <t xml:space="preserve">RFA-DP-27-051</t>
@@ -311,18 +347,6 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/54666d94-e0dc-44d3-90e6-6eb913f79ca9</t>
   </si>
   <si>
-    <t xml:space="preserve">HRSA-27-079</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ryan White HIV/AIDS Program (RWHAP) Integrated HIV/AIDS Planning Resource Allocation Cooperative Agreement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 110 days to deadline · up to $700K (Grants.gov ceiling) · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/a73919b2-7a90-4735-8ec5-a67c08dea3ed</t>
-  </si>
-  <si>
     <t xml:space="preserve">RFA-OH-27-050</t>
   </si>
   <si>
@@ -359,18 +383,6 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/8bb15754-c013-462d-b305-f2a8dd116e08</t>
   </si>
   <si>
-    <t xml:space="preserve">CDC-RFA-PS-27-0239</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Strengthening Services to Prevent the Infectious Disease Consequences of Drug Use</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 236 days to deadline · award not stated on Grants.gov · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/441d2761-0d9c-42ae-a3da-905ce4ed0ca4</t>
-  </si>
-  <si>
     <t xml:space="preserve">HRSA-27-039</t>
   </si>
   <si>
@@ -395,18 +407,6 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/18c0a9f1-fe39-4c7a-8ffd-1d8c656d666f</t>
   </si>
   <si>
-    <t xml:space="preserve">HRSA-27-063</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HIV Care Grant Program - Part B States/Territories Formula and AIDS Drug Assistance Program Formula and AIDS Drug Assistance Program Supplemental Awards</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 92 days to deadline · award not stated on Grants.gov · no cost share → Tier 1: writer can act</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/1d55627c-531e-4a60-95e0-719b256179bf</t>
-  </si>
-  <si>
     <t xml:space="preserve">CDC-RFA-TP22-2201</t>
   </si>
   <si>
@@ -428,67 +428,151 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/42a1b238-2c19-47b4-ae58-f4a775231b78</t>
   </si>
   <si>
+    <t xml:space="preserve">CDC-RFA-DP-27-0043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Statewide Perinatal Quality Collaboratives: Improving Perinatal Care and Outcomes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HHS-CDC-NCCDPHP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 215 days to deadline · about $2.1M per award (estimated: total ÷ expected awards) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needs research and rigorous evaluation, which DHHS reaches only through a partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/477f11ad-e8c7-40ea-84f3-f5bec6e50e3b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HHS-2026-ACF-ORR-ZU-0019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home Study and Post-Release Services for Unaccompanied Alien Children​​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HHS-ACF-ORR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply · partner needed for workforce training and credentialing · 366 days to deadline · up to $100.0M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needs workforce training and credentialing, which DHHS reaches only through a partner; Cooperative agreement with a required evaluation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/cb2cbb9f-741d-4e6b-ad32-557d751f9903</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFA-CK-26-035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emerging Infections Network - Research for Preventing, Detecting, and Managing Travel-associated Infectious Diseases</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply · required capabilities in-house or contracted · 36 days to deadline · up to $6.0M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires funding and monitoring subrecipients; Cooperative agreement with a required evaluation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/10f4a697-e6a1-454a-bb73-74bc933f364a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFA-OH-24-001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National Center for Construction Safety and Health Research and Translation (U54)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply · partner needed for research and rigorous evaluation · 62 days to deadline · up to $5.8M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/b307f2ac-767d-4715-be92-f5326db2cd9d</t>
+  </si>
+  <si>
     <t xml:space="preserve">CDC-RFA-DP-27-0072</t>
   </si>
   <si>
     <t xml:space="preserve">Promoting Population Health through Increased Capacity in Alcohol Epidemiology &amp; the Prevention of Excessive Alcohol Use</t>
   </si>
   <si>
-    <t xml:space="preserve">HHS-CDC-NCCDPHP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 212 days to deadline · award not stated on Grants.gov · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needs research and rigorous evaluation, which DHHS reaches only through a partner</t>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 212 days to deadline · about $1.0M per award (estimated: total ÷ expected awards) · no cost share → Tier 2: needs supervisor or division</t>
   </si>
   <si>
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/6d44bb23-2a1f-4e12-8d72-c2b5b46195d4</t>
   </si>
   <si>
-    <t xml:space="preserve">HHS-2026-ACF-ORR-ZU-0019</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Home Study and Post-Release Services for Unaccompanied Alien Children​​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HHS-ACF-ORR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply · partner needed for workforce training and credentialing · 366 days to deadline · up to $100.0M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needs workforce training and credentialing, which DHHS reaches only through a partner; Cooperative agreement with a required evaluation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/cb2cbb9f-741d-4e6b-ad32-557d751f9903</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RFA-CK-26-035</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emerging Infections Network - Research for Preventing, Detecting, and Managing Travel-associated Infectious Diseases</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply · required capabilities in-house or contracted · 36 days to deadline · up to $6.0M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Requires funding and monitoring subrecipients; Cooperative agreement with a required evaluation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/10f4a697-e6a1-454a-bb73-74bc933f364a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RFA-OH-24-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Center for Construction Safety and Health Research and Translation (U54)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply · partner needed for research and rigorous evaluation · 62 days to deadline · up to $5.8M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/b307f2ac-767d-4715-be92-f5326db2cd9d</t>
+    <t xml:space="preserve">HRSA-27-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiscal Year (FY) 2027 State and Regional Primary Care Association (PCA) Cooperative Agreements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for workforce training and credentialing; partner needed for emergency management · 117 days to deadline · up to $4.9M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needs workforce training and credentialing, which DHHS reaches only through a partner; Needs emergency management, which DHHS reaches only through a partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/88f12b64-0fbc-44ea-a689-57ed9e9fb9dd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RFA-DP-27-036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pilot Testing, Implementation, and Evaluation of the Cervical, Breast and Colorectal Cancer Clinical Decision Support Tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 174 days to deadline · about $3.6M per award (estimated: total ÷ expected awards) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cooperative agreement with a required evaluation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/5686905a-446f-4b0d-8885-e1683d35c3f4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRSA-27-041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rural Communities Opioid Response Program - Evaluation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 174 days to deadline · up to $5.0M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needs research and rigorous evaluation, which DHHS reaches only through a partner; Cooperative agreement with a required evaluation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/44a089ce-dd0a-4cde-b6f4-c77d08d56a08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRSA-27-020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infant-Toddler Court Program–National Resource Center</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for workforce training and credentialing · 203 days to deadline · up to $6.8M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needs workforce training and credentialing, which DHHS reaches only through a partner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/910a75ad-0418-4091-a436-703280874498</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRSA-27-023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Home Visiting Research, Improvement, Sustainability and Evaluation Center (HV-RISE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 146 days to deadline · up to $5.0M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/b9bdeaa2-068f-4aa9-960a-948c0b0a9bfd</t>
   </si>
   <si>
     <t xml:space="preserve">HRSA-27-042</t>
@@ -506,21 +590,6 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/02b2d236-f596-4aca-874d-b8e364156ddc</t>
   </si>
   <si>
-    <t xml:space="preserve">HRSA-27-014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fiscal Year (FY) 2027 State and Regional Primary Care Association (PCA) Cooperative Agreements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for workforce training and credentialing; partner needed for emergency management · 117 days to deadline · up to $4.9M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needs workforce training and credentialing, which DHHS reaches only through a partner; Needs emergency management, which DHHS reaches only through a partner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/88f12b64-0fbc-44ea-a689-57ed9e9fb9dd</t>
-  </si>
-  <si>
     <t xml:space="preserve">CDC-RFA-CE-27-0024</t>
   </si>
   <si>
@@ -539,46 +608,28 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/3c36bc50-73ae-42ad-a727-fae640dad5c9</t>
   </si>
   <si>
-    <t xml:space="preserve">HRSA-27-020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Infant-Toddler Court Program–National Resource Center</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for workforce training and credentialing · 203 days to deadline · up to $6.8M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needs workforce training and credentialing, which DHHS reaches only through a partner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/910a75ad-0418-4091-a436-703280874498</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HRSA-27-041</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rural Communities Opioid Response Program - Evaluation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 174 days to deadline · up to $5.0M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Needs research and rigorous evaluation, which DHHS reaches only through a partner; Cooperative agreement with a required evaluation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/44a089ce-dd0a-4cde-b6f4-c77d08d56a08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HRSA-27-023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Home Visiting Research, Improvement, Sustainability and Evaluation Center (HV-RISE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 146 days to deadline · up to $5.0M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/b9bdeaa2-068f-4aa9-960a-948c0b0a9bfd</t>
+    <t xml:space="preserve">CDC-RFA-PS-27-0011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">National Viral Hepatitis Education, Awareness, and Capacity Building for Communities and Providers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for workforce training and credentialing · 244 days to deadline · about $2.8M per award (estimated: total ÷ expected awards) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/f931e3f2-28c6-4bcb-83ff-894bc6b2266c</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HRSA-27-021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Infant-Toddler Court Program–State Awards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for workforce training and credentialing · 203 days to deadline · up to $700K (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/3fe27753-0c94-4aa0-b7fb-09712631f269</t>
   </si>
   <si>
     <t xml:space="preserve">RFA-OH-27-049</t>
@@ -593,16 +644,46 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/43e32c6d-fbbd-4056-8fd4-f64cdebefd41</t>
   </si>
   <si>
-    <t xml:space="preserve">HRSA-27-021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Infant-Toddler Court Program–State Awards</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for workforce training and credentialing · 203 days to deadline · up to $700K (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/3fe27753-0c94-4aa0-b7fb-09712631f269</t>
+    <t xml:space="preserve">CDC-RFA-CE-27-0039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core State Injury Prevention Program (Core SIPP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 159 days to deadline · about $1.4M per award (estimated: total ÷ expected awards) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/23b80a6d-ae96-4b02-b4ae-69093f8939d5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CDC-RFA-PS-27-0061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demonstration Projects for Whole-Person Health Models for Women Living with HIV in the South</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 166 days to deadline · about $2.5M per award (estimated: total ÷ expected awards) · no cost share → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/06024144-a58a-42d8-8813-75357d9bb7fe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHS-26-MT-144-000-99</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiscal Year 2026 Flood Mitigation Assistance Swift Current</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DHS-DHS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">state agency can apply · required capabilities in-house or contracted · 488 days to deadline · award not stated on Grants.gov · cost share required (25% stated) → Tier 2: needs supervisor or division</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost share required (25% stated): supervisor must approve match</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://simpler.grants.gov/opportunity/4802584e-01a8-4435-9ce9-710fbc85cba0</t>
   </si>
   <si>
     <t xml:space="preserve">RFA-CK-26-036</t>
@@ -614,9 +695,6 @@
     <t xml:space="preserve">state agency can apply · required capabilities in-house or contracted · 36 days to deadline · up to $1.0M (Grants.gov ceiling) · no cost share → Tier 2: needs supervisor or division</t>
   </si>
   <si>
-    <t xml:space="preserve">Cooperative agreement with a required evaluation</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/1a3231f6-36eb-40d1-afe8-232010fa2fe3</t>
   </si>
   <si>
@@ -632,72 +710,6 @@
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/9accc70c-9683-4b78-bb7b-e8fdbcff1b47</t>
   </si>
   <si>
-    <t xml:space="preserve">CDC-RFA-CE-27-0039</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Core State Injury Prevention Program (Core SIPP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 159 days to deadline · award not stated on Grants.gov · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/23b80a6d-ae96-4b02-b4ae-69093f8939d5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RFA-DP-27-036</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pilot Testing, Implementation, and Evaluation of the Cervical, Breast and Colorectal Cancer Clinical Decision Support Tools</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · required capabilities in-house or contracted · 174 days to deadline · award not stated on Grants.gov · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/5686905a-446f-4b0d-8885-e1683d35c3f4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CDC-RFA-PS-27-0011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">National Viral Hepatitis Education, Awareness, and Capacity Building for Communities and Providers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for workforce training and credentialing · 244 days to deadline · award not stated on Grants.gov · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/f931e3f2-28c6-4bcb-83ff-894bc6b2266c</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DHS-26-MT-144-000-99</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fiscal Year 2026 Flood Mitigation Assistance Swift Current</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DHS-DHS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply · required capabilities in-house or contracted · 488 days to deadline · award not stated on Grants.gov · cost share required (25% stated) → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cost share required (25% stated): supervisor must approve match</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/4802584e-01a8-4435-9ce9-710fbc85cba0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CDC-RFA-DP-27-0043</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Statewide Perinatal Quality Collaboratives: Improving Perinatal Care and Outcomes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 215 days to deadline · award not stated on Grants.gov · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/477f11ad-e8c7-40ea-84f3-f5bec6e50e3b</t>
-  </si>
-  <si>
     <t xml:space="preserve">RFA-OH-25-003</t>
   </si>
   <si>
@@ -720,18 +732,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/f2ea8925-6244-47e8-8de5-ffe0007096e7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CDC-RFA-PS-27-0061</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demonstration Projects for Whole-Person Health Models for Women Living with HIV in the South</t>
-  </si>
-  <si>
-    <t xml:space="preserve">state agency can apply, forecast (not yet posted) · partner needed for research and rigorous evaluation · 166 days to deadline · award not stated on Grants.gov · no cost share → Tier 2: needs supervisor or division</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://simpler.grants.gov/opportunity/06024144-a58a-42d8-8813-75357d9bb7fe</t>
   </si>
   <si>
     <t xml:space="preserve">VA-GPD-FORECAST-FY2026-FY2028</t>
@@ -1264,7 +1264,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>14</v>
@@ -1279,10 +1279,10 @@
         <v>17</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>46386</v>
+        <v>46434</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>22024900</v>
+        <v>7500000</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>18</v>
@@ -1320,9 +1320,11 @@
         <v>17</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>46434</v>
-      </c>
-      <c r="J3" s="3"/>
+        <v>46386</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>22024900</v>
+      </c>
       <c r="K3" s="3" t="s">
         <v>24</v>
       </c>
@@ -1353,25 +1355,25 @@
         <v>28</v>
       </c>
       <c r="G4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>46386</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>19182000</v>
+      </c>
+      <c r="K4" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>46391</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>22000000</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>30</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>25</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5">
@@ -1385,25 +1387,25 @@
         <v>4</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="H5" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>46386</v>
+        <v>46391</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>19182000</v>
+        <v>22000000</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>34</v>
@@ -1432,10 +1434,10 @@
         <v>36</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>17</v>
@@ -1450,7 +1452,7 @@
         <v>37</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>38</v>
@@ -1467,7 +1469,7 @@
         <v>6</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>39</v>
@@ -1476,7 +1478,7 @@
         <v>40</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>17</v>
@@ -1491,7 +1493,7 @@
         <v>41</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="M7" s="3" t="s">
         <v>42</v>
@@ -1508,7 +1510,7 @@
         <v>7</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>43</v>
@@ -1523,10 +1525,10 @@
         <v>17</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>46328</v>
+        <v>46398</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>10000000</v>
+        <v>8474576.27118644</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>45</v>
@@ -1549,7 +1551,7 @@
         <v>8</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>47</v>
@@ -1564,16 +1566,16 @@
         <v>17</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>46407</v>
+        <v>46531</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>5149000</v>
+        <v>41250000</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>49</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M9" s="3" t="s">
         <v>50</v>
@@ -1590,7 +1592,7 @@
         <v>9</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>51</v>
@@ -1599,7 +1601,7 @@
         <v>52</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>17</v>
@@ -1608,16 +1610,16 @@
         <v>46387</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>1140000</v>
+        <v>21716666.6666667</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>25</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11">
@@ -1631,34 +1633,34 @@
         <v>10</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E11" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>46328</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="K11" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I11" s="3" t="n">
-        <v>46357</v>
-      </c>
-      <c r="J11" s="3" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>58</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>25</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12">
@@ -1672,13 +1674,13 @@
         <v>11</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E12" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>61</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>23</v>
@@ -1687,19 +1689,19 @@
         <v>17</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>46438</v>
+        <v>46407</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>1000000</v>
+        <v>5149000</v>
       </c>
       <c r="K12" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="L12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="M12" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="13">
@@ -1713,31 +1715,31 @@
         <v>12</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="G13" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="H13" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>46497</v>
+        <v>46477</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>1000000</v>
+        <v>2750000</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>66</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M13" s="3" t="s">
         <v>67</v>
@@ -1754,7 +1756,7 @@
         <v>13</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>68</v>
@@ -1763,20 +1765,22 @@
         <v>69</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>46398</v>
-      </c>
-      <c r="J14" s="3"/>
+        <v>46538</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>3000000</v>
+      </c>
       <c r="K14" s="3" t="s">
         <v>70</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M14" s="3" t="s">
         <v>71</v>
@@ -1793,7 +1797,7 @@
         <v>14</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="E15" s="3" t="s">
         <v>72</v>
@@ -1802,16 +1806,16 @@
         <v>73</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>46464</v>
+        <v>46503</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>750000</v>
+        <v>2217391.30434783</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>74</v>
@@ -1834,7 +1838,7 @@
         <v>15</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>76</v>
@@ -1849,14 +1853,16 @@
         <v>17</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>46477</v>
-      </c>
-      <c r="J16" s="3"/>
+        <v>46387</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>1140000</v>
+      </c>
       <c r="K16" s="3" t="s">
         <v>79</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M16" s="3" t="s">
         <v>80</v>
@@ -1882,23 +1888,21 @@
         <v>82</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="3" t="n">
-        <v>46503</v>
-      </c>
+      <c r="I17" s="3"/>
       <c r="J17" s="3"/>
       <c r="K17" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M17" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18">
@@ -1912,13 +1916,13 @@
         <v>17</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>23</v>
@@ -1927,17 +1931,19 @@
         <v>17</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>46538</v>
-      </c>
-      <c r="J18" s="3"/>
+        <v>46357</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>1000000</v>
+      </c>
       <c r="K18" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19">
@@ -1951,27 +1957,31 @@
         <v>18</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>91</v>
+        <v>16</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
+      <c r="I19" s="3" t="n">
+        <v>46438</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>1000000</v>
+      </c>
       <c r="K19" s="3" t="s">
         <v>92</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>93</v>
@@ -1988,7 +1998,7 @@
         <v>19</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>94</v>
@@ -1997,22 +2007,22 @@
         <v>95</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>46468</v>
+        <v>46497</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>725000</v>
+        <v>1000000</v>
       </c>
       <c r="K20" s="3" t="s">
         <v>96</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M20" s="3" t="s">
         <v>97</v>
@@ -2029,7 +2039,7 @@
         <v>20</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>98</v>
@@ -2038,16 +2048,16 @@
         <v>99</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>46405</v>
+        <v>46464</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>700000</v>
+        <v>750000</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>100</v>
@@ -2070,7 +2080,7 @@
         <v>21</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>102</v>
@@ -2079,22 +2089,22 @@
         <v>103</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>46386</v>
+        <v>46405</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>685000</v>
+        <v>700000</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>104</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>105</v>
@@ -2111,7 +2121,7 @@
         <v>22</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>106</v>
@@ -2120,22 +2130,22 @@
         <v>107</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>46466</v>
+        <v>46468</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>650000</v>
+        <v>725000</v>
       </c>
       <c r="K23" s="3" t="s">
         <v>108</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M23" s="3" t="s">
         <v>109</v>
@@ -2152,7 +2162,7 @@
         <v>23</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>110</v>
@@ -2161,16 +2171,16 @@
         <v>111</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>46462</v>
+        <v>46386</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>500000</v>
+        <v>685000</v>
       </c>
       <c r="K24" s="3" t="s">
         <v>112</v>
@@ -2208,14 +2218,16 @@
         <v>17</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>46531</v>
-      </c>
-      <c r="J25" s="3"/>
+        <v>46466</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>650000</v>
+      </c>
       <c r="K25" s="3" t="s">
         <v>116</v>
       </c>
       <c r="L25" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="M25" s="3" t="s">
         <v>117</v>
@@ -2232,7 +2244,7 @@
         <v>25</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E26" s="3" t="s">
         <v>118</v>
@@ -2241,13 +2253,13 @@
         <v>119</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>46532</v>
+        <v>46462</v>
       </c>
       <c r="J26" s="3" t="n">
         <v>500000</v>
@@ -2256,7 +2268,7 @@
         <v>120</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="M26" s="3" t="s">
         <v>121</v>
@@ -2273,7 +2285,7 @@
         <v>26</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>122</v>
@@ -2282,22 +2294,22 @@
         <v>123</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>46508</v>
+        <v>46532</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>300000</v>
+        <v>500000</v>
       </c>
       <c r="K27" s="3" t="s">
         <v>124</v>
       </c>
       <c r="L27" s="3" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="M27" s="3" t="s">
         <v>125</v>
@@ -2314,7 +2326,7 @@
         <v>27</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>126</v>
@@ -2323,20 +2335,22 @@
         <v>127</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>46387</v>
-      </c>
-      <c r="J28" s="3"/>
+        <v>46508</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>300000</v>
+      </c>
       <c r="K28" s="3" t="s">
         <v>128</v>
       </c>
       <c r="L28" s="3" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="M28" s="3" t="s">
         <v>129</v>
@@ -2394,7 +2408,7 @@
         <v>2</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>137</v>
@@ -2409,9 +2423,11 @@
         <v>17</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>46507</v>
-      </c>
-      <c r="J30" s="3"/>
+        <v>46510</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>2141025.64102564</v>
+      </c>
       <c r="K30" s="3" t="s">
         <v>140</v>
       </c>
@@ -2483,7 +2499,7 @@
         <v>150</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>133</v>
@@ -2524,7 +2540,7 @@
         <v>155</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>53</v>
+        <v>78</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>133</v>
@@ -2565,25 +2581,25 @@
         <v>159</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>16</v>
+        <v>139</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>46483</v>
+        <v>46507</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>500000</v>
+        <v>1002916.66666667</v>
       </c>
       <c r="K34" s="3" t="s">
         <v>160</v>
       </c>
       <c r="L34" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="M34" s="3" t="s">
         <v>161</v>
-      </c>
-      <c r="M34" s="3" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="35">
@@ -2600,13 +2616,13 @@
         <v>58</v>
       </c>
       <c r="E35" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F35" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="F35" s="3" t="s">
-        <v>164</v>
-      </c>
       <c r="G35" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>17</v>
@@ -2618,13 +2634,13 @@
         <v>4900000</v>
       </c>
       <c r="K35" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="L35" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="L35" s="3" t="s">
+      <c r="M35" s="3" t="s">
         <v>166</v>
-      </c>
-      <c r="M35" s="3" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="36">
@@ -2641,31 +2657,31 @@
         <v>58</v>
       </c>
       <c r="E36" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F36" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="G36" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>46469</v>
+      </c>
+      <c r="J36" s="3" t="n">
+        <v>3625000</v>
+      </c>
+      <c r="K36" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="G36" s="3" t="s">
+      <c r="L36" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="H36" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I36" s="3" t="n">
-        <v>46494</v>
-      </c>
-      <c r="J36" s="3" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="K36" s="3" t="s">
+      <c r="M36" s="3" t="s">
         <v>171</v>
-      </c>
-      <c r="L36" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="M36" s="3" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="37">
@@ -2679,34 +2695,34 @@
         <v>9</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E37" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>46469</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="K37" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="L37" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="G37" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I37" s="3" t="n">
-        <v>46498</v>
-      </c>
-      <c r="J37" s="3" t="n">
-        <v>6750000</v>
-      </c>
-      <c r="K37" s="3" t="s">
+      <c r="M37" s="3" t="s">
         <v>176</v>
-      </c>
-      <c r="L37" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="M37" s="3" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="38">
@@ -2723,31 +2739,31 @@
         <v>57</v>
       </c>
       <c r="E38" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>46498</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>6750000</v>
+      </c>
+      <c r="K38" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="L38" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="G38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I38" s="3" t="n">
-        <v>46469</v>
-      </c>
-      <c r="J38" s="3" t="n">
-        <v>5000000</v>
-      </c>
-      <c r="K38" s="3" t="s">
+      <c r="M38" s="3" t="s">
         <v>181</v>
-      </c>
-      <c r="L38" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="M38" s="3" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="39">
@@ -2764,13 +2780,13 @@
         <v>56</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>17</v>
@@ -2782,13 +2798,13 @@
         <v>5000000</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="L39" s="3" t="s">
         <v>141</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="40">
@@ -2802,34 +2818,34 @@
         <v>12</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E40" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>46483</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>500000</v>
+      </c>
+      <c r="K40" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="L40" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="G40" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I40" s="3" t="n">
-        <v>46444</v>
-      </c>
-      <c r="J40" s="3" t="n">
-        <v>1400000</v>
-      </c>
-      <c r="K40" s="3" t="s">
+      <c r="M40" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="L40" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="M40" s="3" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="41">
@@ -2843,34 +2859,34 @@
         <v>13</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E41" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="F41" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="G41" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="G41" s="3" t="s">
-        <v>16</v>
-      </c>
       <c r="H41" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>46498</v>
+        <v>46494</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>700000</v>
+        <v>1200000</v>
       </c>
       <c r="K41" s="3" t="s">
         <v>194</v>
       </c>
       <c r="L41" s="3" t="s">
-        <v>177</v>
+        <v>195</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="42">
@@ -2884,31 +2900,31 @@
         <v>14</v>
       </c>
       <c r="D42" s="3" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>133</v>
+        <v>17</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>46331</v>
+        <v>46539</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>1000000</v>
+        <v>2750000</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>199</v>
+        <v>180</v>
       </c>
       <c r="M42" s="3" t="s">
         <v>200</v>
@@ -2925,7 +2941,7 @@
         <v>15</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>201</v>
@@ -2934,22 +2950,22 @@
         <v>202</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>46455</v>
+        <v>46498</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>900000</v>
+        <v>700000</v>
       </c>
       <c r="K43" s="3" t="s">
         <v>203</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>141</v>
+        <v>180</v>
       </c>
       <c r="M43" s="3" t="s">
         <v>204</v>
@@ -2966,7 +2982,7 @@
         <v>16</v>
       </c>
       <c r="D44" s="3" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>205</v>
@@ -2975,20 +2991,22 @@
         <v>206</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>170</v>
+        <v>78</v>
       </c>
       <c r="H44" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>46454</v>
-      </c>
-      <c r="J44" s="3"/>
+        <v>46444</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>1400000</v>
+      </c>
       <c r="K44" s="3" t="s">
         <v>207</v>
       </c>
       <c r="L44" s="3" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="M44" s="3" t="s">
         <v>208</v>
@@ -3005,7 +3023,7 @@
         <v>17</v>
       </c>
       <c r="D45" s="3" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E45" s="3" t="s">
         <v>209</v>
@@ -3014,20 +3032,22 @@
         <v>210</v>
       </c>
       <c r="G45" s="3" t="s">
-        <v>53</v>
+        <v>193</v>
       </c>
       <c r="H45" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>46469</v>
-      </c>
-      <c r="J45" s="3"/>
+        <v>46454</v>
+      </c>
+      <c r="J45" s="3" t="n">
+        <v>1423076.92307692</v>
+      </c>
       <c r="K45" s="3" t="s">
         <v>211</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="M45" s="3" t="s">
         <v>212</v>
@@ -3044,7 +3064,7 @@
         <v>18</v>
       </c>
       <c r="D46" s="3" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E46" s="3" t="s">
         <v>213</v>
@@ -3053,20 +3073,22 @@
         <v>214</v>
       </c>
       <c r="G46" s="3" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="H46" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>46539</v>
-      </c>
-      <c r="J46" s="3"/>
+        <v>46461</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>2500000</v>
+      </c>
       <c r="K46" s="3" t="s">
         <v>215</v>
       </c>
       <c r="L46" s="3" t="s">
-        <v>177</v>
+        <v>195</v>
       </c>
       <c r="M46" s="3" t="s">
         <v>216</v>
@@ -3122,7 +3144,7 @@
         <v>20</v>
       </c>
       <c r="D48" s="3" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>223</v>
@@ -3131,20 +3153,22 @@
         <v>224</v>
       </c>
       <c r="G48" s="3" t="s">
-        <v>139</v>
+        <v>78</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>17</v>
+        <v>133</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>46510</v>
-      </c>
-      <c r="J48" s="3"/>
+        <v>46331</v>
+      </c>
+      <c r="J48" s="3" t="n">
+        <v>1000000</v>
+      </c>
       <c r="K48" s="3" t="s">
         <v>225</v>
       </c>
       <c r="L48" s="3" t="s">
-        <v>141</v>
+        <v>170</v>
       </c>
       <c r="M48" s="3" t="s">
         <v>226</v>
@@ -3161,7 +3185,7 @@
         <v>21</v>
       </c>
       <c r="D49" s="3" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E49" s="3" t="s">
         <v>227</v>
@@ -3170,22 +3194,22 @@
         <v>228</v>
       </c>
       <c r="G49" s="3" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>133</v>
+        <v>17</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>47052</v>
+        <v>46455</v>
       </c>
       <c r="J49" s="3" t="n">
-        <v>550000</v>
+        <v>900000</v>
       </c>
       <c r="K49" s="3" t="s">
         <v>229</v>
       </c>
       <c r="L49" s="3" t="s">
-        <v>177</v>
+        <v>141</v>
       </c>
       <c r="M49" s="3" t="s">
         <v>230</v>
@@ -3202,7 +3226,7 @@
         <v>22</v>
       </c>
       <c r="D50" s="3" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E50" s="3" t="s">
         <v>231</v>
@@ -3211,22 +3235,22 @@
         <v>232</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>170</v>
+        <v>78</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>17</v>
+        <v>133</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>46510</v>
+        <v>47052</v>
       </c>
       <c r="J50" s="3" t="n">
-        <v>450000</v>
+        <v>550000</v>
       </c>
       <c r="K50" s="3" t="s">
         <v>233</v>
       </c>
       <c r="L50" s="3" t="s">
-        <v>152</v>
+        <v>180</v>
       </c>
       <c r="M50" s="3" t="s">
         <v>234</v>
@@ -3243,7 +3267,7 @@
         <v>23</v>
       </c>
       <c r="D51" s="3" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="E51" s="3" t="s">
         <v>235</v>
@@ -3252,20 +3276,22 @@
         <v>236</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>23</v>
+        <v>193</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>17</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>46461</v>
-      </c>
-      <c r="J51" s="3"/>
+        <v>46510</v>
+      </c>
+      <c r="J51" s="3" t="n">
+        <v>450000</v>
+      </c>
       <c r="K51" s="3" t="s">
         <v>237</v>
       </c>
       <c r="L51" s="3" t="s">
-        <v>172</v>
+        <v>152</v>
       </c>
       <c r="M51" s="3" t="s">
         <v>238</v>
@@ -3369,7 +3395,7 @@
         <v>252</v>
       </c>
       <c r="G54" s="3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="H54" s="3" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
Fix wording, takeaway styling and stale takeaways; final checks
</commit_message>
<xml_diff>
--- a/docs/downloads/top_results.xlsx
+++ b/docs/downloads/top_results.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="403">
   <si>
-    <t xml:space="preserve">Our tool sorted grant opportunities into three tiers, instead of a singular list. These tiers are differentiated by the level of authority needed from a grant coordinator's perspective. Tier 1 grants can be directly acted upon by the grant writer using the tool. Tier 2 opportunities would need approval by a supervisor. Tier 3 grants, due to high matching costs or other factors, need oversight from upper legislature. The 3 tiers allow a user to make desicions about opportunities based on their capabilities and their priorities. Furthermore, within the tiers, the grants are sorted based on an "impact score" which is calculated with multiple metrics, including plan fit with the agency, people reached, population reached, help per person, and award size. While the weights for these metrics were equal, a user of our tool can adjust these weights according to their priorities. Also, there are a few opportunities chosen for the DMVA on this list, to showcase the generalizability of our model.</t>
+    <t xml:space="preserve">Our tool sorted grant opportunities into three tiers, instead of a singular list. These tiers are differentiated by the level of authority needed from a grant coordinator's perspective. Tier 1 grants can be directly acted upon by the grant writer using the tool. Tier 2 opportunities would need approval by a supervisor. Tier 3 grants, due to high matching costs or other factors, need approval from the secretary or the legislature. The 3 tiers allow a user to make decisions about opportunities based on their capabilities and their priorities. Furthermore, within the tiers, the grants are sorted based on an "impact score" which is calculated with multiple metrics, including plan fit with the agency's strategic plan, people reached, help per person, award size, and program priorities. While the weights for these metrics were equal, a user of our tool can adjust these weights according to their priorities. Also, there are a few opportunities chosen for the DMVA on this list, to showcase the generalizability of our model.</t>
   </si>
   <si>
     <t xml:space="preserve">How these results were ranked:</t>
@@ -1133,7 +1133,7 @@
     <t xml:space="preserve">HHS-ACF</t>
   </si>
   <si>
-    <t xml:space="preserve">Top ranked in Tier 3 for strong plan fit and a large award (up to $15M), funding statewide early care, education data and technology infrastructure, but its 30% match and required state designation need the secretary.</t>
+    <t xml:space="preserve">Top ranked in Tier 3 for strong plan fit and a large award (up to $15M), funding statewide early care and education data and technology infrastructure, but its 30% match and required state designation need the secretary.</t>
   </si>
   <si>
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/8d272419-96d1-4898-9706-0d86a1e63c03</t>
@@ -1199,7 +1199,7 @@
     <t xml:space="preserve">VA-CSHF</t>
   </si>
   <si>
-    <t xml:space="preserve">Top ranked for DMVA strong plan fit, the highest help per veteran (about $444), and funding construction and modernization of State Veterans Homes, but needs a 35% state match and an appropriation.</t>
+    <t xml:space="preserve">Top ranked for DMVA for strong plan fit, the highest help per veteran (about $444), and funding construction and modernization of State Veterans Homes, but needs a 35% state match and an appropriation.</t>
   </si>
   <si>
     <t xml:space="preserve">https://simpler.grants.gov/opportunity/59462b36-6d05-4832-a628-427f72260f3d</t>

</xml_diff>